<commit_message>
Refresh integration handoffs from validated source snapshots
</commit_message>
<xml_diff>
--- a/Website/static/downloads/integrations/events/EventRegister.xlsx
+++ b/Website/static/downloads/integrations/events/EventRegister.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <x:si>
     <x:t>Event register</x:t>
   </x:si>
@@ -31,12 +31,24 @@
     <x:t>Level</x:t>
   </x:si>
   <x:si>
+    <x:t>Computer</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Log</x:t>
+  </x:si>
+  <x:si>
     <x:t>Message</x:t>
   </x:si>
   <x:si>
     <x:t>Demo.Backup</x:t>
   </x:si>
   <x:si>
+    <x:t>DEMO-SRV01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Application</x:t>
+  </x:si>
+  <x:si>
     <x:t>The overnight backup did not complete.</x:t>
   </x:si>
   <x:si>
@@ -46,10 +58,16 @@
     <x:t>Demo.Inventory</x:t>
   </x:si>
   <x:si>
+    <x:t>DEMO-SRV02</x:t>
+  </x:si>
+  <x:si>
     <x:t>The inventory queue is above its warning threshold.</x:t>
   </x:si>
   <x:si>
     <x:t>Demo.Sync</x:t>
+  </x:si>
+  <x:si>
+    <x:t>System</x:t>
   </x:si>
   <x:si>
     <x:t>Synchronization completed after a retry.</x:t>
@@ -116,14 +134,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventRegister" displayName="EventRegister" ref="A4:E8" headerRowCount="1" totalsRowShown="0">
-  <x:autoFilter ref="A4:E8"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventRegister" displayName="EventRegister" ref="A4:G8" headerRowCount="1" totalsRowShown="0">
+  <x:autoFilter ref="A4:G8"/>
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="TimeCreated"/>
     <x:tableColumn id="2" name="EventId"/>
     <x:tableColumn id="3" name="Provider"/>
     <x:tableColumn id="4" name="Level"/>
-    <x:tableColumn id="5" name="Message"/>
+    <x:tableColumn id="5" name="Computer"/>
+    <x:tableColumn id="6" name="Log"/>
+    <x:tableColumn id="7" name="Message"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -131,14 +151,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G8"/>
   <x:sheetFormatPr xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="70" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -167,6 +189,12 @@
       <c r="E4" t="s">
         <v>6</v>
       </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="n">
@@ -176,13 +204,19 @@
         <v>1001</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D5" s="7">
         <v>2</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -193,13 +227,19 @@
         <v>1001</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D6" s="7">
         <v>2</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -210,13 +250,19 @@
         <v>2004</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D7" s="7">
         <v>3</v>
       </c>
       <c r="E7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>11</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
@@ -227,13 +273,19 @@
         <v>3002</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D8" s="7">
         <v>3</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh integration downloads with precise prices and timestamps
</commit_message>
<xml_diff>
--- a/Website/static/downloads/integrations/events/EventRegister.xlsx
+++ b/Website/static/downloads/integrations/events/EventRegister.xlsx
@@ -77,9 +77,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm"/>
     <x:numFmt numFmtId="165" formatCode="[h]:mm:ss"/>
+    <x:numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm:ss.000"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -111,14 +112,15 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -154,7 +156,7 @@
   <dimension ref="A1:G8"/>
   <x:sheetFormatPr xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
@@ -197,94 +199,94 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="7" t="n">
         <v>46306.34027777778</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="8">
         <v>1001</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="8">
         <v>2</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>46306.34166666667</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="8">
         <v>1001</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="8">
         <v>2</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>46306.34583333333</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="8">
         <v>2004</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="8">
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>46306.350694444445</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="8">
         <v>3002</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="8">
         <v>3</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="8" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Explain reporting workflows through embedded PowerShell articles
</commit_message>
<xml_diff>
--- a/Website/static/downloads/integrations/events/EventRegister.xlsx
+++ b/Website/static/downloads/integrations/events/EventRegister.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
-  <x:si>
-    <x:t>Event register</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Synthetic incident exercise / 11 October 2026</x:t>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+  <x:si>
+    <x:t>Windows event register</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Application log | last 24 hours | levels 1, 2, 3 | limit 100 | collected 2026-10-11 06:30:00 +02:00</x:t>
   </x:si>
   <x:si>
     <x:t>TimeCreated</x:t>
@@ -43,34 +43,31 @@
     <x:t>Demo.Backup</x:t>
   </x:si>
   <x:si>
-    <x:t>DEMO-SRV01</x:t>
+    <x:t>server-a</x:t>
   </x:si>
   <x:si>
     <x:t>Application</x:t>
   </x:si>
   <x:si>
-    <x:t>The overnight backup did not complete.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>The backup retry did not complete.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Demo.Inventory</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DEMO-SRV02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>The inventory queue is above its warning threshold.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Demo.Sync</x:t>
-  </x:si>
-  <x:si>
-    <x:t>System</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Synchronization completed after a retry.</x:t>
+    <x:t>Backup task failed while writing the local archive. Inspect the task log and available space.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>The next backup attempt is waiting for the prior task to finish.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Demo.Service</x:t>
+  </x:si>
+  <x:si>
+    <x:t>server-b</x:t>
+  </x:si>
+  <x:si>
+    <x:t>The reporting service could not open its configured input file. Inspect its service account and file permissions.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Demo.Storage</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Available space is below the configured warning threshold.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -82,7 +79,7 @@
     <x:numFmt numFmtId="165" formatCode="[h]:mm:ss"/>
     <x:numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm:ss.000"/>
   </x:numFmts>
-  <x:fonts count="3">
+  <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Calibri"/>
@@ -91,11 +88,6 @@
       <x:b/>
       <x:sz val="11"/>
       <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="2">
@@ -112,10 +104,9 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -166,7 +157,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -198,96 +189,96 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="7" t="n">
-        <v>46306.34027777778</v>
-      </c>
-      <c r="B5" s="8">
-        <v>1001</v>
-      </c>
-      <c r="C5" s="8" t="s">
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>46306.23625</v>
+      </c>
+      <c r="B5" s="7">
+        <v>101</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="7">
         <v>2</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="8" t="s">
+      <c r="F5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="7" t="n">
-        <v>46306.34166666667</v>
-      </c>
-      <c r="B6" s="8">
-        <v>1001</v>
-      </c>
-      <c r="C6" s="8" t="s">
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>46306.23752314815</v>
+      </c>
+      <c r="B6" s="7">
+        <v>102</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
+        <v>3</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>46306.252291666664</v>
+      </c>
+      <c r="B7" s="7">
+        <v>301</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="7">
         <v>2</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="7" t="n">
-        <v>46306.34583333333</v>
-      </c>
-      <c r="B7" s="8">
-        <v>2004</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="8">
+      <c r="E7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>46306.254270833335</v>
+      </c>
+      <c r="B8" s="7">
+        <v>401</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="7">
         <v>3</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="7" t="n">
-        <v>46306.350694444445</v>
-      </c>
-      <c r="B8" s="8">
-        <v>3002</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="8">
-        <v>3</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>18</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate integration downloads with the current commands
</commit_message>
<xml_diff>
--- a/Website/static/downloads/integrations/events/EventRegister.xlsx
+++ b/Website/static/downloads/integrations/events/EventRegister.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:bookViews xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:bookViews>
     <x:workbookView/>
   </x:bookViews>
-  <sheets>
-    <sheet name="Events" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" r:id="R90d03f6fab4246f1"/>
+  </x:sheets>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -82,12 +82,12 @@
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
-      <x:name val="Calibri"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:name val="Calibri"/>
+      <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
   <x:fills count="2">
@@ -142,6 +142,289 @@
 </x:table>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="OfficeIMO Modern">
+  <a:themeElements>
+    <a:clrScheme name="Modern">
+      <a:dk1>
+        <a:srgbClr val="1B2433"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="5B6575"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="F6F8FB"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="3F64D7"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="DC7536"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="058E80"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="A52758"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="3F2F6B"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="255319"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="3F64D7"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="A52758"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Modern">
+      <a:majorFont>
+        <a:latin typeface="Aptos"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G8"/>

</xml_diff>